<commit_message>
Improve BRVM financial validation and 2025 reports
</commit_message>
<xml_diff>
--- a/data/brvm_financials_2020_2025.xlsx
+++ b/data/brvm_financials_2020_2025.xlsx
@@ -826,14 +826,10 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>fy=2019 pub=2020 title=AIR LIQUIDE CI : Etats financiers exercice 2019 [score=60]; fy=2019 pub=2020 title=AIR LIQUIDE CI : Etats financiers exercice 2019 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>0</v>
       </c>
@@ -1718,16 +1714,16 @@
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="n">
-        <v>0.4132825127489414</v>
+        <v>0.4132825127489415</v>
       </c>
       <c r="T19" t="n">
         <v>0.3921530221106811</v>
       </c>
       <c r="U19" t="n">
-        <v>0.1711151817717444</v>
+        <v>0.1711151817717445</v>
       </c>
       <c r="V19" t="n">
-        <v>0.0208437925592222</v>
+        <v>0.02084379255922226</v>
       </c>
       <c r="W19" t="n">
         <v>7.209407250890875</v>
@@ -2566,22 +2562,22 @@
       </c>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="n">
-        <v>0.2477694941473889</v>
+        <v>0.247769494147389</v>
       </c>
       <c r="T31" t="n">
         <v>0.291638423204646</v>
       </c>
       <c r="U31" t="n">
-        <v>0.2224226416019503</v>
+        <v>0.2224226416019504</v>
       </c>
       <c r="V31" t="n">
-        <v>0.0186723189941644</v>
+        <v>0.01867231899416446</v>
       </c>
       <c r="W31" t="n">
         <v>10.9118916976227</v>
       </c>
       <c r="X31" t="n">
-        <v>0.0839497222930236</v>
+        <v>0.08394972229302365</v>
       </c>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr">
@@ -2900,14 +2896,10 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>fy=2021 pub=2022 title=BOA NIGER : États financiers exercice 2021 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
         <v>0</v>
       </c>
@@ -3353,7 +3345,7 @@
         <v>0.2471761772040487</v>
       </c>
       <c r="V43" t="n">
-        <v>0.0279695546194774</v>
+        <v>0.02796955461947743</v>
       </c>
       <c r="W43" t="n">
         <v>7.837329752541723</v>
@@ -4065,43 +4057,61 @@
       <c r="B55" t="n">
         <v>2025</v>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
+      <c r="C55" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=BERNABE CÔTE D'IVOIRE : Etats financiers - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>BERNABE CI : Etats financiers - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260430_-_etats_financiers_-_exercice_2025_-_bernabe_ci.pdf</t>
+        </is>
+      </c>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="L55" t="n">
+        <v>2318122</v>
+      </c>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
+      <c r="N55" t="n">
+        <v>7769953951</v>
+      </c>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
+      <c r="Q55" t="n">
+        <v>1260999614</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1887953177</v>
+      </c>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="inlineStr"/>
-      <c r="U55" t="inlineStr"/>
+      <c r="U55" t="n">
+        <v>0.0002983443678841437</v>
+      </c>
       <c r="V55" t="inlineStr"/>
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr"/>
-      <c r="Y55" t="inlineStr"/>
+      <c r="Y55" t="n">
+        <v>0.6679189025247738</v>
+      </c>
       <c r="Z55" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/bernabe-ci</t>
@@ -4531,7 +4541,7 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -4552,18 +4562,12 @@
       <c r="M61" t="n">
         <v>68063</v>
       </c>
-      <c r="N61" t="n">
-        <v>120570</v>
-      </c>
+      <c r="N61" t="inlineStr"/>
       <c r="O61" t="n">
-        <v>1126270</v>
-      </c>
-      <c r="P61" t="n">
-        <v>1005700</v>
-      </c>
-      <c r="Q61" t="n">
-        <v>44542</v>
-      </c>
+        <v>1015578</v>
+      </c>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr"/>
       <c r="S61" t="n">
         <v>0.4226819270381852</v>
@@ -4571,18 +4575,12 @@
       <c r="T61" t="n">
         <v>0.3853194834197728</v>
       </c>
-      <c r="U61" t="n">
-        <v>0.2175167952226922</v>
-      </c>
+      <c r="U61" t="inlineStr"/>
       <c r="V61" t="n">
-        <v>0.0232857130173049</v>
-      </c>
-      <c r="W61" t="n">
-        <v>8.341212573608692</v>
-      </c>
-      <c r="X61" t="n">
-        <v>0.1070524829747751</v>
-      </c>
+        <v>0.02582371811914004</v>
+      </c>
+      <c r="W61" t="inlineStr"/>
+      <c r="X61" t="inlineStr"/>
       <c r="Y61" t="inlineStr"/>
       <c r="Z61" t="inlineStr">
         <is>
@@ -5316,14 +5314,10 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>fy=2023 pub=2024 title=AFRICA GLOBAL LOGISTICS CI (ex AFRICA GLOBAL LOGISTICS CI ) : Etats financiers - Exercice 2023 [score=60]; fy=2022 pub=2023 title=AFRICA GLOBAL LOGISTICS CI (ex BOLLORE) : Etats financiers - exercice 2022 [score=60]; fy=2022 pub=2023 title=AFRICA GLOBAL LOGISTICS CI (ex BOLLORE) : Etats financiers exercice 2022 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="n">
         <v>0</v>
       </c>
@@ -6186,14 +6180,10 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>fy=2021 pub=2022 title=CIE : Etats financiers IFRS exercice 2021 [score=60]; fy=2021 pub=2022 title=CIE : Etats financiers SYSCOHADA exercice 2021 [score=60]; fy=2023 pub=2024 title=CIE CI : Etats financiers - Exercice 2023 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
         <v>0</v>
       </c>
@@ -6525,36 +6515,54 @@
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
-          <t>missing_report</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
+          <t>partial_core_metrics</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>fy=2022 pub=2023 title=CORIS BANK INTERNATIONAL BURKINA FASO : Etats financiers Exercice 2022 [score=60]</t>
+          <t>core_metrics_count=3; report=CORIS BANK INTERNATIONAL BF : Rapport d'activités annuel - Exercice 2025</t>
         </is>
       </c>
       <c r="H91" t="n">
-        <v>0</v>
-      </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>CORIS BANK INTERNATIONAL BF : Rapport d'activités annuel - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/fr/coris-bank-international-bf-rapport-dactivites-annuel-exercice-2025</t>
+        </is>
+      </c>
       <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
+      <c r="L91" t="n">
+        <v>65495000000000</v>
+      </c>
+      <c r="M91" t="n">
+        <v>138986000000000</v>
+      </c>
       <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
+      <c r="O91" t="n">
+        <v>2997779000000000</v>
+      </c>
       <c r="P91" t="inlineStr"/>
       <c r="Q91" t="inlineStr"/>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="inlineStr"/>
-      <c r="T91" t="inlineStr"/>
+      <c r="T91" t="n">
+        <v>0.4712345128286302</v>
+      </c>
       <c r="U91" t="inlineStr"/>
-      <c r="V91" t="inlineStr"/>
+      <c r="V91" t="n">
+        <v>0.02184784135188084</v>
+      </c>
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="inlineStr"/>
       <c r="Y91" t="inlineStr"/>
@@ -7268,14 +7276,10 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>fy=2019 pub=2020 title=CROWN SIEM CI : Etats Financiers - Exercice 2019 [score=60]; fy=2022 pub=None title=CROWN SIEM CI : Etats financiers - Exercice 2022 [score=60]; fy=2020 pub=2021 title=CROWN SIEM CI : Etats financiers - exercice 2020 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
       <c r="H103" t="n">
         <v>0</v>
       </c>
@@ -7983,36 +7987,50 @@
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>fy=2019 pub=2020 title=ECOBANK CI : Etats financiers Exercice 2019 [score=60]; fy=2020 pub=2021 title=ECOBANK CI : Etats financiers exercice 2020 [score=60]; fy=2022 pub=2023 title=ECOBANK CI : Etats financiers exercice 2022 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
       <c r="H115" t="n">
-        <v>0</v>
-      </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>ECOBANK CI : Rapport d'activités et Etats financiers - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/fr/ecobank-ci-rapport-dactivites-et-etats-financiers-exercice-2025</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>73995</v>
+      </c>
+      <c r="L115" t="n">
+        <v>63482</v>
+      </c>
+      <c r="M115" t="n">
+        <v>132725</v>
+      </c>
       <c r="N115" t="inlineStr"/>
-      <c r="O115" t="inlineStr"/>
+      <c r="O115" t="n">
+        <v>2054491</v>
+      </c>
       <c r="P115" t="inlineStr"/>
       <c r="Q115" t="inlineStr"/>
       <c r="R115" t="inlineStr"/>
-      <c r="S115" t="inlineStr"/>
-      <c r="T115" t="inlineStr"/>
+      <c r="S115" t="n">
+        <v>0.5575061216801658</v>
+      </c>
+      <c r="T115" t="n">
+        <v>0.4782972311169712</v>
+      </c>
       <c r="U115" t="inlineStr"/>
-      <c r="V115" t="inlineStr"/>
+      <c r="V115" t="n">
+        <v>0.03089913754793766</v>
+      </c>
       <c r="W115" t="inlineStr"/>
       <c r="X115" t="inlineStr"/>
       <c r="Y115" t="inlineStr"/>
@@ -8403,44 +8421,56 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="n">
+        <v>6</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>ETI TG : Etats financiers IFRS - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260413_-_etats_financiers_ifrs_-_exercice_2025_-_eti_tg.pdf</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="L121" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="M121" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="N121" t="n">
+        <v>2863000</v>
+      </c>
+      <c r="O121" t="n">
+        <v>34487000</v>
+      </c>
+      <c r="P121" t="n">
+        <v>31624000</v>
+      </c>
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="n">
         <v>4</v>
       </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>ETI TG : Etats financiers IFRS - Exercice 2025</t>
-        </is>
-      </c>
-      <c r="J121" t="inlineStr">
-        <is>
-          <t>https://www.brvm.org/sites/default/files/20260413_-_etats_financiers_ifrs_-_exercice_2025_-_eti_tg.pdf</t>
-        </is>
-      </c>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="n">
-        <v>594.122</v>
-      </c>
-      <c r="M121" t="n">
-        <v>17</v>
-      </c>
-      <c r="N121" t="n">
-        <v>60</v>
-      </c>
-      <c r="O121" t="inlineStr"/>
-      <c r="P121" t="inlineStr"/>
-      <c r="Q121" t="n">
-        <v>422.321</v>
-      </c>
-      <c r="R121" t="inlineStr"/>
-      <c r="S121" t="inlineStr"/>
       <c r="T121" t="n">
-        <v>34.94835294117647</v>
+        <v>3</v>
       </c>
       <c r="U121" t="n">
-        <v>9.902033333333332</v>
-      </c>
-      <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr"/>
-      <c r="X121" t="inlineStr"/>
+        <v>2.09570380719525</v>
+      </c>
+      <c r="V121" t="n">
+        <v>0.1739786006321223</v>
+      </c>
+      <c r="W121" t="n">
+        <v>11.04575619979043</v>
+      </c>
+      <c r="X121" t="n">
+        <v>0.08301678893496101</v>
+      </c>
       <c r="Y121" t="inlineStr"/>
       <c r="Z121" t="inlineStr">
         <is>
@@ -11235,39 +11265,61 @@
       <c r="B175" t="n">
         <v>2025</v>
       </c>
-      <c r="C175" t="inlineStr"/>
-      <c r="D175" t="inlineStr"/>
+      <c r="C175" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=LOTERIE NATIONALE DU BENIN : Etats financiers - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
       <c r="H175" t="n">
-        <v>0</v>
-      </c>
-      <c r="I175" t="inlineStr"/>
-      <c r="J175" t="inlineStr"/>
-      <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
-      <c r="M175" t="inlineStr"/>
-      <c r="N175" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>LNB BN : Etats financiers - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260430_-_etats_financiers_-_exercice_2025_-_lnb_bn.pdf</t>
+        </is>
+      </c>
+      <c r="K175" t="n">
+        <v>6376159291</v>
+      </c>
+      <c r="L175" t="n">
+        <v>4622243779</v>
+      </c>
+      <c r="M175" t="n">
+        <v>98598057859</v>
+      </c>
+      <c r="N175" t="n">
+        <v>21953860132</v>
+      </c>
       <c r="O175" t="inlineStr"/>
       <c r="P175" t="inlineStr"/>
       <c r="Q175" t="inlineStr"/>
-      <c r="R175" t="inlineStr"/>
-      <c r="S175" t="inlineStr"/>
-      <c r="T175" t="inlineStr"/>
-      <c r="U175" t="inlineStr"/>
+      <c r="R175" t="n">
+        <v>9661311921</v>
+      </c>
+      <c r="S175" t="n">
+        <v>0.06466820370963307</v>
+      </c>
+      <c r="T175" t="n">
+        <v>0.04687966354885035</v>
+      </c>
+      <c r="U175" t="n">
+        <v>0.2105435559490791</v>
+      </c>
       <c r="V175" t="inlineStr"/>
       <c r="W175" t="inlineStr"/>
       <c r="X175" t="inlineStr"/>
@@ -11556,14 +11608,10 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>fy=2019 pub=2020 title=MOVIS CÔTE D'IVOIRE : Etats financiers – Exercice 2019 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr"/>
       <c r="H181" t="n">
         <v>0</v>
       </c>
@@ -12092,7 +12140,7 @@
         <v>1631946812</v>
       </c>
       <c r="S187" t="n">
-        <v>0.235988240880043</v>
+        <v>0.2359882408800431</v>
       </c>
       <c r="T187" t="n">
         <v>0.396291974618772</v>
@@ -12497,38 +12545,62 @@
       <c r="B193" t="n">
         <v>2025</v>
       </c>
-      <c r="C193" t="inlineStr"/>
-      <c r="D193" t="inlineStr"/>
+      <c r="C193" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>missing_report</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>nearest_report_is_different_fiscal_year</t>
+          <t>partial_core_metrics</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>fy=2024 pub=2025 title=NESTLE CÔTE D'IVOIRE : Etats financiers - Exercice 2024 (Annule et remplace le précédent) [score=60]; fy=2024 pub=2025 title=NESTLE CI : Etats financiers - Exercice 2024 [score=60]</t>
+          <t>core_metrics_count=3; report=NESTLE CI - Etats financiers - Exercice 2025</t>
         </is>
       </c>
       <c r="H193" t="n">
-        <v>0</v>
-      </c>
-      <c r="I193" t="inlineStr"/>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>NESTLE CI - Etats financiers - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260430_-_etats_financiers_-_exercice_2025_-_nestle_ci.pdf</t>
+        </is>
+      </c>
+      <c r="K193" t="n">
+        <v>37.687</v>
+      </c>
+      <c r="L193" t="n">
+        <v>18.426</v>
+      </c>
+      <c r="M193" t="n">
+        <v>233.261</v>
+      </c>
       <c r="N193" t="inlineStr"/>
       <c r="O193" t="inlineStr"/>
       <c r="P193" t="inlineStr"/>
       <c r="Q193" t="inlineStr"/>
       <c r="R193" t="inlineStr"/>
-      <c r="S193" t="inlineStr"/>
-      <c r="T193" t="inlineStr"/>
+      <c r="S193" t="n">
+        <v>0.1615657996836162</v>
+      </c>
+      <c r="T193" t="n">
+        <v>0.07899305927694728</v>
+      </c>
       <c r="U193" t="inlineStr"/>
       <c r="V193" t="inlineStr"/>
       <c r="W193" t="inlineStr"/>
@@ -13257,40 +13329,60 @@
       <c r="B205" t="n">
         <v>2025</v>
       </c>
-      <c r="C205" t="inlineStr"/>
-      <c r="D205" t="inlineStr"/>
+      <c r="C205" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F205" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=NSIA BANQUE CÔTE D'IVOIRE : Etats financiers certifiés par les Commissaires Aux Comptes - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr"/>
+      <c r="G205" t="inlineStr"/>
       <c r="H205" t="n">
-        <v>0</v>
-      </c>
-      <c r="I205" t="inlineStr"/>
-      <c r="J205" t="inlineStr"/>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="inlineStr"/>
-      <c r="M205" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>NSIA BANQUE CI : Etats financiers et Communiqué - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260513_-_etats_financiers_et_communique_-_exercice_2025_-_nsia_banque_ci.pdf</t>
+        </is>
+      </c>
+      <c r="K205" t="n">
+        <v>39937000000</v>
+      </c>
+      <c r="L205" t="n">
+        <v>38112000000</v>
+      </c>
+      <c r="M205" t="n">
+        <v>31000000000</v>
+      </c>
       <c r="N205" t="inlineStr"/>
-      <c r="O205" t="inlineStr"/>
+      <c r="O205" t="n">
+        <v>2510429000000</v>
+      </c>
       <c r="P205" t="inlineStr"/>
       <c r="Q205" t="inlineStr"/>
       <c r="R205" t="inlineStr"/>
-      <c r="S205" t="inlineStr"/>
-      <c r="T205" t="inlineStr"/>
+      <c r="S205" t="n">
+        <v>1.288290322580645</v>
+      </c>
+      <c r="T205" t="n">
+        <v>1.22941935483871</v>
+      </c>
       <c r="U205" t="inlineStr"/>
-      <c r="V205" t="inlineStr"/>
+      <c r="V205" t="n">
+        <v>0.0151814689839864</v>
+      </c>
       <c r="W205" t="inlineStr"/>
       <c r="X205" t="inlineStr"/>
       <c r="Y205" t="inlineStr"/>
@@ -13765,7 +13857,7 @@
       <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I211" t="inlineStr">
         <is>
@@ -13786,17 +13878,13 @@
       <c r="M211" t="n">
         <v>146176657128</v>
       </c>
-      <c r="N211" t="n">
-        <v>57541603762</v>
-      </c>
+      <c r="N211" t="inlineStr"/>
       <c r="O211" t="n">
-        <v>826786578374</v>
-      </c>
-      <c r="P211" t="n">
-        <v>205659518733</v>
-      </c>
+        <v>8.267865783746161e+23</v>
+      </c>
+      <c r="P211" t="inlineStr"/>
       <c r="Q211" t="n">
-        <v>82298442903</v>
+        <v>-1</v>
       </c>
       <c r="R211" t="n">
         <v>147863552993</v>
@@ -13805,22 +13893,16 @@
         <v>0.1755767003039766</v>
       </c>
       <c r="T211" t="n">
-        <v>0.1086830241171035</v>
-      </c>
-      <c r="U211" t="n">
-        <v>0.2760945144614059</v>
-      </c>
+        <v>0.1086830241171036</v>
+      </c>
+      <c r="U211" t="inlineStr"/>
       <c r="V211" t="n">
-        <v>0.0192152625206422</v>
-      </c>
-      <c r="W211" t="n">
-        <v>3.574101263907</v>
-      </c>
-      <c r="X211" t="n">
-        <v>0.06959668343330409</v>
-      </c>
+        <v>1.921526252062797e-14</v>
+      </c>
+      <c r="W211" t="inlineStr"/>
+      <c r="X211" t="inlineStr"/>
       <c r="Y211" t="n">
-        <v>0.5565836965036007</v>
+        <v>-6.762991824275594e-12</v>
       </c>
       <c r="Z211" t="inlineStr">
         <is>
@@ -14024,7 +14106,7 @@
         <v>0.0863144076140466</v>
       </c>
       <c r="U214" t="n">
-        <v>1.823625842213696e-07</v>
+        <v>1.823625842213697e-07</v>
       </c>
       <c r="V214" t="inlineStr"/>
       <c r="W214" t="inlineStr"/>
@@ -14189,42 +14271,64 @@
       <c r="B217" t="n">
         <v>2025</v>
       </c>
-      <c r="C217" t="inlineStr"/>
-      <c r="D217" t="inlineStr"/>
+      <c r="C217" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F217" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G217" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=ORAGROUP TOGO : Etats financiers - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr"/>
+      <c r="G217" t="inlineStr"/>
       <c r="H217" t="n">
-        <v>0</v>
-      </c>
-      <c r="I217" t="inlineStr"/>
-      <c r="J217" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>ORAGROUP TG : Etats financiers - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260504_-_etats_financiers_-_exercice_2025_-_oragroup_tg.pdf</t>
+        </is>
+      </c>
       <c r="K217" t="inlineStr"/>
-      <c r="L217" t="inlineStr"/>
+      <c r="L217" t="n">
+        <v>21643</v>
+      </c>
       <c r="M217" t="inlineStr"/>
-      <c r="N217" t="inlineStr"/>
-      <c r="O217" t="inlineStr"/>
-      <c r="P217" t="inlineStr"/>
+      <c r="N217" t="n">
+        <v>113165</v>
+      </c>
+      <c r="O217" t="n">
+        <v>4014192</v>
+      </c>
+      <c r="P217" t="n">
+        <v>3901027</v>
+      </c>
       <c r="Q217" t="inlineStr"/>
       <c r="R217" t="inlineStr"/>
       <c r="S217" t="inlineStr"/>
       <c r="T217" t="inlineStr"/>
-      <c r="U217" t="inlineStr"/>
-      <c r="V217" t="inlineStr"/>
-      <c r="W217" t="inlineStr"/>
-      <c r="X217" t="inlineStr"/>
+      <c r="U217" t="n">
+        <v>0.1912517121017983</v>
+      </c>
+      <c r="V217" t="n">
+        <v>0.005391620530358289</v>
+      </c>
+      <c r="W217" t="n">
+        <v>34.47202757036186</v>
+      </c>
+      <c r="X217" t="n">
+        <v>0.02819122752474221</v>
+      </c>
       <c r="Y217" t="inlineStr"/>
       <c r="Z217" t="inlineStr">
         <is>
@@ -14255,7 +14359,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>fy=2023 pub=2024 title=ORANGE CI : Etats financiers - Exercice 2023 [score=60]; fy=2025 pub=2026 title=ORANGE CI : Etats financiers - Exercice 2025 [score=60]; fy=2022 pub=2023 title=ORANGE CI : Etats financiers Consolidés exercice 2022 [score=60]</t>
+          <t>fy=2023 pub=2024 title=ORANGE CI : Etats financiers - Exercice 2023 [score=260]; fy=2024 pub=2025 title=ORANGE CI : Etats financiers - Exercice 2024 [score=260]; fy=2025 pub=2026 title=ORANGE CI : Etats financiers - Exercice 2025 [score=260]</t>
         </is>
       </c>
       <c r="H218" t="n">
@@ -14307,7 +14411,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>fy=2022 pub=2023 title=ORANGE CI : Etats financiers Consolidés exercice 2022 [score=60]</t>
+          <t>fy=2022 pub=2023 title=ORANGE CI : Etats financiers consolides exercice 2022 [score=260]</t>
         </is>
       </c>
       <c r="H219" t="n">
@@ -14361,11 +14465,11 @@
       <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>ORANGE CI : Etats financiers Consolidés exercice 2022</t>
+          <t>ORANGE CI : Etats financiers consolides exercice 2022</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
@@ -14382,20 +14486,16 @@
       <c r="M220" t="n">
         <v>965025</v>
       </c>
-      <c r="N220" t="n">
-        <v>642547</v>
-      </c>
+      <c r="N220" t="inlineStr"/>
       <c r="O220" t="n">
         <v>2017757</v>
       </c>
-      <c r="P220" t="n">
-        <v>329078</v>
-      </c>
+      <c r="P220" t="inlineStr"/>
       <c r="Q220" t="n">
-        <v>399056</v>
+        <v>9</v>
       </c>
       <c r="R220" t="n">
-        <v>329078</v>
+        <v>2811</v>
       </c>
       <c r="S220" t="n">
         <v>0.2702872982565218</v>
@@ -14403,20 +14503,14 @@
       <c r="T220" t="n">
         <v>0.1590476930649465</v>
       </c>
-      <c r="U220" t="n">
-        <v>0.2388696857973035</v>
-      </c>
+      <c r="U220" t="inlineStr"/>
       <c r="V220" t="n">
         <v>0.07606713791601261</v>
       </c>
-      <c r="W220" t="n">
-        <v>0.5121461931967622</v>
-      </c>
-      <c r="X220" t="n">
-        <v>0.318446175629672</v>
-      </c>
+      <c r="W220" t="inlineStr"/>
+      <c r="X220" t="inlineStr"/>
       <c r="Y220" t="n">
-        <v>1.212648672958994</v>
+        <v>0.0032017075773745</v>
       </c>
       <c r="Z220" t="inlineStr">
         <is>
@@ -14449,7 +14543,7 @@
       <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I221" t="inlineStr">
         <is>
@@ -14462,50 +14556,36 @@
         </is>
       </c>
       <c r="K221" t="n">
-        <v>258</v>
+        <v>257960</v>
       </c>
       <c r="L221" t="n">
-        <v>154.9</v>
+        <v>154890</v>
       </c>
       <c r="M221" t="n">
-        <v>1016.5</v>
-      </c>
-      <c r="N221" t="n">
-        <v>627178</v>
-      </c>
+        <v>1016532965025</v>
+      </c>
+      <c r="N221" t="inlineStr"/>
       <c r="O221" t="n">
         <v>2074719</v>
       </c>
-      <c r="P221" t="n">
-        <v>526703</v>
-      </c>
+      <c r="P221" t="inlineStr"/>
       <c r="Q221" t="n">
-        <v>475016</v>
-      </c>
-      <c r="R221" t="n">
-        <v>526703</v>
-      </c>
+        <v>993769</v>
+      </c>
+      <c r="R221" t="inlineStr"/>
       <c r="S221" t="n">
-        <v>0.2538121003443187</v>
+        <v>2.537645200651766e-07</v>
       </c>
       <c r="T221" t="n">
-        <v>0.1523856369896704</v>
-      </c>
-      <c r="U221" t="n">
-        <v>0.0002469793264432</v>
-      </c>
+        <v>1.523708579349325e-07</v>
+      </c>
+      <c r="U221" t="inlineStr"/>
       <c r="V221" t="n">
-        <v>7.466071308933885e-05</v>
-      </c>
-      <c r="W221" t="n">
-        <v>0.8397982709852705</v>
-      </c>
-      <c r="X221" t="n">
-        <v>0.3022953951836369</v>
-      </c>
-      <c r="Y221" t="n">
-        <v>0.9018668965242272</v>
-      </c>
+        <v>0.0746558931595073</v>
+      </c>
+      <c r="W221" t="inlineStr"/>
+      <c r="X221" t="inlineStr"/>
+      <c r="Y221" t="inlineStr"/>
       <c r="Z221" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/orange-ci</t>
@@ -14537,11 +14617,11 @@
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>ORANGE CÔTE D'IVOIRE : Etats financiers - Exercice 2024</t>
+          <t>ORANGE CI : Etats financiers - Exercice 2024</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
@@ -14550,28 +14630,22 @@
         </is>
       </c>
       <c r="K222" t="n">
-        <v>263.2</v>
+        <v>263200000000</v>
       </c>
       <c r="L222" t="n">
-        <v>158.2</v>
+        <v>158200000000</v>
       </c>
       <c r="M222" t="n">
-        <v>1084.1</v>
+        <v>1084100000000</v>
       </c>
       <c r="N222" t="n">
-        <v>713.8</v>
-      </c>
-      <c r="O222" t="n">
-        <v>2309.1</v>
-      </c>
-      <c r="P222" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="Q222" t="n">
-        <v>5.5</v>
-      </c>
+        <v>713800000000</v>
+      </c>
+      <c r="O222" t="inlineStr"/>
+      <c r="P222" t="inlineStr"/>
+      <c r="Q222" t="inlineStr"/>
       <c r="R222" t="n">
-        <v>6.3</v>
+        <v>1304300000000</v>
       </c>
       <c r="S222" t="n">
         <v>0.2427820311779356</v>
@@ -14582,18 +14656,10 @@
       <c r="U222" t="n">
         <v>0.2216307088820397</v>
       </c>
-      <c r="V222" t="n">
-        <v>0.0685115412931445</v>
-      </c>
-      <c r="W222" t="n">
-        <v>0.0088260016811431</v>
-      </c>
-      <c r="X222" t="n">
-        <v>0.3091247672253259</v>
-      </c>
-      <c r="Y222" t="n">
-        <v>0.873015873015873</v>
-      </c>
+      <c r="V222" t="inlineStr"/>
+      <c r="W222" t="inlineStr"/>
+      <c r="X222" t="inlineStr"/>
+      <c r="Y222" t="inlineStr"/>
       <c r="Z222" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/orange-ci</t>
@@ -14638,28 +14704,28 @@
         </is>
       </c>
       <c r="K223" t="n">
-        <v>287.2</v>
+        <v>287200000000</v>
       </c>
       <c r="L223" t="n">
-        <v>167.8</v>
+        <v>167800000000</v>
       </c>
       <c r="M223" t="n">
-        <v>1197.1</v>
+        <v>1197100000000</v>
       </c>
       <c r="N223" t="n">
-        <v>707.8</v>
+        <v>707800000000</v>
       </c>
       <c r="O223" t="n">
-        <v>2554.1</v>
+        <v>2554100000000</v>
       </c>
       <c r="P223" t="n">
-        <v>6.3</v>
+        <v>1846300000000</v>
       </c>
       <c r="Q223" t="n">
-        <v>5.5</v>
+        <v>1436100000000</v>
       </c>
       <c r="R223" t="n">
-        <v>6.3</v>
+        <v>1520200000000</v>
       </c>
       <c r="S223" t="n">
         <v>0.2399131233815053</v>
@@ -14671,16 +14737,16 @@
         <v>0.2370726193840068</v>
       </c>
       <c r="V223" t="n">
-        <v>0.0656982890254884</v>
+        <v>0.06569828902548842</v>
       </c>
       <c r="W223" t="n">
-        <v>0.008900819440519901</v>
+        <v>2.608505227465386</v>
       </c>
       <c r="X223" t="n">
         <v>0.2771230570455346</v>
       </c>
       <c r="Y223" t="n">
-        <v>0.873015873015873</v>
+        <v>0.9446783317984476</v>
       </c>
       <c r="Z223" t="inlineStr">
         <is>
@@ -15117,7 +15183,7 @@
       <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr"/>
       <c r="H229" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I229" t="inlineStr">
         <is>
@@ -15130,50 +15196,36 @@
         </is>
       </c>
       <c r="K229" t="n">
-        <v>18163004</v>
+        <v>19393765</v>
       </c>
       <c r="L229" t="n">
-        <v>15508655</v>
+        <v>15861643</v>
       </c>
       <c r="M229" t="n">
-        <v>197629996</v>
-      </c>
-      <c r="N229" t="n">
-        <v>142638984</v>
-      </c>
+        <v>996172</v>
+      </c>
+      <c r="N229" t="inlineStr"/>
       <c r="O229" t="n">
-        <v>199116293</v>
-      </c>
-      <c r="P229" t="n">
-        <v>56477309</v>
-      </c>
+        <v>-85706070</v>
+      </c>
+      <c r="P229" t="inlineStr"/>
       <c r="Q229" t="n">
-        <v>86256798</v>
-      </c>
-      <c r="R229" t="n">
-        <v>41633570</v>
-      </c>
+        <v>93705506</v>
+      </c>
+      <c r="R229" t="inlineStr"/>
       <c r="S229" t="n">
-        <v>0.0919040852482737</v>
+        <v>19.46828961263718</v>
       </c>
       <c r="T229" t="n">
-        <v>0.0784731837974636</v>
-      </c>
-      <c r="U229" t="n">
-        <v>0.1087266227302909</v>
-      </c>
+        <v>15.92259469248282</v>
+      </c>
+      <c r="U229" t="inlineStr"/>
       <c r="V229" t="n">
-        <v>0.077887423305937</v>
-      </c>
-      <c r="W229" t="n">
-        <v>0.3959458166078917</v>
-      </c>
-      <c r="X229" t="n">
-        <v>0.7163601825391557</v>
-      </c>
-      <c r="Y229" t="n">
-        <v>2.071808831190792</v>
-      </c>
+        <v>-0.1850702406492329</v>
+      </c>
+      <c r="W229" t="inlineStr"/>
+      <c r="X229" t="inlineStr"/>
+      <c r="Y229" t="inlineStr"/>
       <c r="Z229" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/palm-ci</t>
@@ -16341,7 +16393,7 @@
       <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr"/>
       <c r="H247" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I247" t="inlineStr">
         <is>
@@ -16360,44 +16412,30 @@
         <v>24972070150</v>
       </c>
       <c r="M247" t="n">
-        <v>340830548704</v>
-      </c>
-      <c r="N247" t="n">
-        <v>8649304155</v>
-      </c>
+        <v>3.408305487042794e+23</v>
+      </c>
+      <c r="N247" t="inlineStr"/>
       <c r="O247" t="n">
-        <v>96555131405</v>
-      </c>
-      <c r="P247" t="n">
-        <v>87905827250</v>
-      </c>
+        <v>2.258427356442222e+23</v>
+      </c>
+      <c r="P247" t="inlineStr"/>
       <c r="Q247" t="n">
-        <v>1016146221799</v>
-      </c>
-      <c r="R247" t="n">
-        <v>36225398864</v>
-      </c>
+        <v>101614627795</v>
+      </c>
+      <c r="R247" t="inlineStr"/>
       <c r="S247" t="n">
-        <v>0.11188586618777</v>
+        <v>1.118858661876784e-13</v>
       </c>
       <c r="T247" t="n">
-        <v>0.0732682860880742</v>
-      </c>
-      <c r="U247" t="n">
-        <v>2.887176783529357</v>
-      </c>
+        <v>7.32682860880142e-14</v>
+      </c>
+      <c r="U247" t="inlineStr"/>
       <c r="V247" t="n">
-        <v>0.2586301710393286</v>
-      </c>
-      <c r="W247" t="n">
-        <v>10.16334096647339</v>
-      </c>
-      <c r="X247" t="n">
-        <v>0.0895789175483645</v>
-      </c>
-      <c r="Y247" t="n">
-        <v>28.05065654663705</v>
-      </c>
+        <v>1.105728288260702e-13</v>
+      </c>
+      <c r="W247" t="inlineStr"/>
+      <c r="X247" t="inlineStr"/>
+      <c r="Y247" t="inlineStr"/>
       <c r="Z247" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/saph-ci</t>
@@ -17182,10 +17220,10 @@
         <v>0.1015662579719731</v>
       </c>
       <c r="U259" t="n">
-        <v>0.1015295807378525</v>
+        <v>0.1015295807378526</v>
       </c>
       <c r="V259" t="n">
-        <v>0.07775509249263721</v>
+        <v>0.07775509249263722</v>
       </c>
       <c r="W259" t="n">
         <v>0.3057611724591109</v>
@@ -17674,16 +17712,16 @@
       <c r="S265" t="inlineStr"/>
       <c r="T265" t="inlineStr"/>
       <c r="U265" t="n">
-        <v>-0.2706631609043969</v>
+        <v>-0.270663160904397</v>
       </c>
       <c r="V265" t="n">
-        <v>-0.0177284201678543</v>
+        <v>-0.01772842016785431</v>
       </c>
       <c r="W265" t="n">
         <v>14.26719010164094</v>
       </c>
       <c r="X265" t="n">
-        <v>0.0654999376664942</v>
+        <v>0.06549993766649426</v>
       </c>
       <c r="Y265" t="n">
         <v>0.7988803957067786</v>
@@ -17989,35 +18027,51 @@
       <c r="D271" t="inlineStr"/>
       <c r="E271" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F271" t="inlineStr">
-        <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G271" t="inlineStr">
-        <is>
-          <t>fy=2019 pub=2020 title=SOCIETE GENERALE CI : Etats financiers certifiés et approuvés exercice 2019 [score=95]; fy=2019 pub=2020 title=SOCIETE GENERALE CI : Etats financiers certifiés et approuvés exercice 2019 (Annule et remplace le précédent) [score=95]; fy=2019 pub=2020 title=SOCIETE GENERALE CI : Etats financiers exercice 2019 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr"/>
+      <c r="G271" t="inlineStr"/>
       <c r="H271" t="n">
-        <v>0</v>
-      </c>
-      <c r="I271" t="inlineStr"/>
-      <c r="J271" t="inlineStr"/>
-      <c r="K271" t="inlineStr"/>
-      <c r="L271" t="inlineStr"/>
-      <c r="M271" t="inlineStr"/>
-      <c r="N271" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>SOCIETE GENERALE CI : Rapport d'activités annuel et Etats Financiers - Exercice 2025 - (Annule et remplace le précédent)</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/fr/societe-generale-ci-rapport-dactivites-annuel-et-etats-financiers-exercice-2025-annule-et-remplace</t>
+        </is>
+      </c>
+      <c r="K271" t="n">
+        <v>15000000000</v>
+      </c>
+      <c r="L271" t="n">
+        <v>0</v>
+      </c>
+      <c r="M271" t="n">
+        <v>4900000000</v>
+      </c>
+      <c r="N271" t="n">
+        <v>451721000000000</v>
+      </c>
       <c r="O271" t="inlineStr"/>
       <c r="P271" t="inlineStr"/>
-      <c r="Q271" t="inlineStr"/>
+      <c r="Q271" t="n">
+        <v>37061000000000</v>
+      </c>
       <c r="R271" t="inlineStr"/>
-      <c r="S271" t="inlineStr"/>
-      <c r="T271" t="inlineStr"/>
-      <c r="U271" t="inlineStr"/>
+      <c r="S271" t="n">
+        <v>3.061224489795918</v>
+      </c>
+      <c r="T271" t="n">
+        <v>0</v>
+      </c>
+      <c r="U271" t="n">
+        <v>0</v>
+      </c>
       <c r="V271" t="inlineStr"/>
       <c r="W271" t="inlineStr"/>
       <c r="X271" t="inlineStr"/>
@@ -18333,36 +18387,50 @@
       <c r="D277" t="inlineStr"/>
       <c r="E277" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F277" t="inlineStr">
-        <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G277" t="inlineStr">
-        <is>
-          <t>fy=2020 pub=2021 title=SIB CI : Etats financiers certifiés et approuvés - exercice 2020 [score=95]; fy=2019 pub=2020 title=SIB CI : Etats financiers exercice 2019 [score=60]; fy=2020 pub=2021 title=SIB CÔTE D'IVOIRE : Etats Financiers - Exercice 2020 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr"/>
+      <c r="G277" t="inlineStr"/>
       <c r="H277" t="n">
-        <v>0</v>
-      </c>
-      <c r="I277" t="inlineStr"/>
-      <c r="J277" t="inlineStr"/>
-      <c r="K277" t="inlineStr"/>
-      <c r="L277" t="inlineStr"/>
-      <c r="M277" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>SIB CI  : Rapport d'activités annuel et Etats Financiers - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/fr/sib-ci-rapport-dactivites-annuel-et-etats-financiers-exercice-2025</t>
+        </is>
+      </c>
+      <c r="K277" t="n">
+        <v>57440</v>
+      </c>
+      <c r="L277" t="n">
+        <v>50234</v>
+      </c>
+      <c r="M277" t="n">
+        <v>102763108663</v>
+      </c>
       <c r="N277" t="inlineStr"/>
-      <c r="O277" t="inlineStr"/>
+      <c r="O277" t="n">
+        <v>1685249</v>
+      </c>
       <c r="P277" t="inlineStr"/>
       <c r="Q277" t="inlineStr"/>
       <c r="R277" t="inlineStr"/>
-      <c r="S277" t="inlineStr"/>
-      <c r="T277" t="inlineStr"/>
+      <c r="S277" t="n">
+        <v>5.589554534435893e-07</v>
+      </c>
+      <c r="T277" t="n">
+        <v>4.88833012679061e-07</v>
+      </c>
       <c r="U277" t="inlineStr"/>
-      <c r="V277" t="inlineStr"/>
+      <c r="V277" t="n">
+        <v>0.02980805803771431</v>
+      </c>
       <c r="W277" t="inlineStr"/>
       <c r="X277" t="inlineStr"/>
       <c r="Y277" t="inlineStr"/>
@@ -18759,7 +18827,7 @@
       <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr"/>
       <c r="H283" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I283" t="inlineStr">
         <is>
@@ -18780,42 +18848,28 @@
       <c r="M283" t="n">
         <v>21263067001</v>
       </c>
-      <c r="N283" t="n">
-        <v>758352000</v>
-      </c>
+      <c r="N283" t="inlineStr"/>
       <c r="O283" t="n">
         <v>21455050944</v>
       </c>
-      <c r="P283" t="n">
-        <v>12469506200</v>
-      </c>
+      <c r="P283" t="inlineStr"/>
       <c r="Q283" t="n">
-        <v>1607854647</v>
-      </c>
-      <c r="R283" t="n">
-        <v>8643081002</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="R283" t="inlineStr"/>
       <c r="S283" t="n">
-        <v>0.106494884622877</v>
+        <v>0.1064948846228771</v>
       </c>
       <c r="T283" t="n">
-        <v>0.08016017369083391</v>
-      </c>
-      <c r="U283" t="n">
-        <v>2.247572557334852</v>
-      </c>
+        <v>0.08016017369083396</v>
+      </c>
+      <c r="U283" t="inlineStr"/>
       <c r="V283" t="n">
-        <v>0.0794428849620912</v>
-      </c>
-      <c r="W283" t="n">
-        <v>16.44290013080997</v>
-      </c>
-      <c r="X283" t="n">
-        <v>0.0353460824669855</v>
-      </c>
-      <c r="Y283" t="n">
-        <v>0.1860279507536657</v>
-      </c>
+        <v>0.07944288496209129</v>
+      </c>
+      <c r="W283" t="inlineStr"/>
+      <c r="X283" t="inlineStr"/>
+      <c r="Y283" t="inlineStr"/>
       <c r="Z283" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/sicable</t>
@@ -19172,14 +19226,10 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G289" t="inlineStr">
-        <is>
-          <t>fy=2020 pub=2023 title=SICOR CI : Etats financiers - Exercice 2020 [score=60]; fy=2021 pub=2023 title=SICOR CI : Etats financiers - Exercice 2021 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr"/>
       <c r="H289" t="n">
         <v>0</v>
       </c>
@@ -19903,40 +19953,56 @@
       <c r="B301" t="n">
         <v>2025</v>
       </c>
-      <c r="C301" t="inlineStr"/>
-      <c r="D301" t="inlineStr"/>
+      <c r="C301" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F301" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G301" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=SITAB CÔTE D'IVOIRE : Etats financiers - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr"/>
+      <c r="G301" t="inlineStr"/>
       <c r="H301" t="n">
-        <v>0</v>
-      </c>
-      <c r="I301" t="inlineStr"/>
-      <c r="J301" t="inlineStr"/>
-      <c r="K301" t="inlineStr"/>
-      <c r="L301" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>SITAB CI : Etats financiers SYSCOHADA - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260430_-_etats_financiers_syscohada_-_exercice_2025_-_sitab_ci.pdf</t>
+        </is>
+      </c>
+      <c r="K301" t="n">
+        <v>57068888519</v>
+      </c>
+      <c r="L301" t="n">
+        <v>44173762491</v>
+      </c>
       <c r="M301" t="inlineStr"/>
       <c r="N301" t="inlineStr"/>
-      <c r="O301" t="inlineStr"/>
+      <c r="O301" t="n">
+        <v>94925572191</v>
+      </c>
       <c r="P301" t="inlineStr"/>
-      <c r="Q301" t="inlineStr"/>
+      <c r="Q301" t="n">
+        <v>36157775979</v>
+      </c>
       <c r="R301" t="inlineStr"/>
       <c r="S301" t="inlineStr"/>
       <c r="T301" t="inlineStr"/>
       <c r="U301" t="inlineStr"/>
-      <c r="V301" t="inlineStr"/>
+      <c r="V301" t="n">
+        <v>0.4653515535531127</v>
+      </c>
       <c r="W301" t="inlineStr"/>
       <c r="X301" t="inlineStr"/>
       <c r="Y301" t="inlineStr"/>
@@ -20389,40 +20455,62 @@
       <c r="B307" t="n">
         <v>2025</v>
       </c>
-      <c r="C307" t="inlineStr"/>
-      <c r="D307" t="inlineStr"/>
+      <c r="C307" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F307" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G307" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=SMB CÔTE D'IVOIRE : Etats financiers - Exercice 2024 [score=60]; fy=2024 pub=2025 title=SMB CÔTE D'IVOIRE : Etats financiers - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr"/>
       <c r="H307" t="n">
-        <v>0</v>
-      </c>
-      <c r="I307" t="inlineStr"/>
-      <c r="J307" t="inlineStr"/>
-      <c r="K307" t="inlineStr"/>
-      <c r="L307" t="inlineStr"/>
-      <c r="M307" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>SMB CI : Etats financiers et projet d'affectation du résultat - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260512_-_etats_financiers_et_projet_daffectation_du_resultat_-_exercice_2025_-_smb_ci.pdf</t>
+        </is>
+      </c>
+      <c r="K307" t="n">
+        <v>17828</v>
+      </c>
+      <c r="L307" t="n">
+        <v>13075</v>
+      </c>
+      <c r="M307" t="n">
+        <v>206740</v>
+      </c>
       <c r="N307" t="inlineStr"/>
-      <c r="O307" t="inlineStr"/>
+      <c r="O307" t="n">
+        <v>180003163113</v>
+      </c>
       <c r="P307" t="inlineStr"/>
-      <c r="Q307" t="inlineStr"/>
+      <c r="Q307" t="n">
+        <v>128963134430</v>
+      </c>
       <c r="R307" t="inlineStr"/>
-      <c r="S307" t="inlineStr"/>
-      <c r="T307" t="inlineStr"/>
+      <c r="S307" t="n">
+        <v>0.08623391699719454</v>
+      </c>
+      <c r="T307" t="n">
+        <v>0.06324368772371095</v>
+      </c>
       <c r="U307" t="inlineStr"/>
-      <c r="V307" t="inlineStr"/>
+      <c r="V307" t="n">
+        <v>7.263761243902113e-08</v>
+      </c>
       <c r="W307" t="inlineStr"/>
       <c r="X307" t="inlineStr"/>
       <c r="Y307" t="inlineStr"/>
@@ -21174,46 +21262,46 @@
         </is>
       </c>
       <c r="K319" t="n">
-        <v>9105153</v>
+        <v>9105153000000000</v>
       </c>
       <c r="L319" t="n">
-        <v>4662738</v>
+        <v>4662738000000000</v>
       </c>
       <c r="M319" t="n">
-        <v>189429713</v>
+        <v>1.89429713e+17</v>
       </c>
       <c r="N319" t="n">
-        <v>3134154</v>
+        <v>3134154000000000</v>
       </c>
       <c r="O319" t="n">
-        <v>472671520</v>
+        <v>4.7267152e+17</v>
       </c>
       <c r="P319" t="n">
-        <v>452955725</v>
+        <v>4.52955725e+17</v>
       </c>
       <c r="Q319" t="n">
-        <v>454</v>
+        <v>454000000000</v>
       </c>
       <c r="R319" t="n">
-        <v>307017158</v>
+        <v>3.07017158e+17</v>
       </c>
       <c r="S319" t="n">
-        <v>0.048066128886549</v>
+        <v>0.04806612888654907</v>
       </c>
       <c r="T319" t="n">
-        <v>0.0246146073187578</v>
+        <v>0.02461460731875785</v>
       </c>
       <c r="U319" t="n">
         <v>1.487718216781945</v>
       </c>
       <c r="V319" t="n">
-        <v>0.009864647652136901</v>
+        <v>0.009864647652136942</v>
       </c>
       <c r="W319" t="n">
         <v>144.5224851746277</v>
       </c>
       <c r="X319" t="n">
-        <v>0.0066307231711358</v>
+        <v>0.006630723171135845</v>
       </c>
       <c r="Y319" t="n">
         <v>1.478744715629216e-06</v>
@@ -21692,13 +21780,13 @@
       <c r="S325" t="inlineStr"/>
       <c r="T325" t="inlineStr"/>
       <c r="U325" t="n">
-        <v>-0.9685469744340228</v>
+        <v>-0.9685469744340229</v>
       </c>
       <c r="V325" t="n">
         <v>-1.024871417538472</v>
       </c>
       <c r="W325" t="n">
-        <v>-0.0549575704235452</v>
+        <v>-0.05495757042354528</v>
       </c>
       <c r="X325" t="n">
         <v>1.058153548140877</v>
@@ -22198,10 +22286,18 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr"/>
-      <c r="G332" t="inlineStr"/>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>partial_core_metrics</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>core_metrics_count=2; report=SONATEL SENEGAL : Résultats financiers 2020 (Annule et remplace le précédent)</t>
+        </is>
+      </c>
       <c r="H332" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I332" t="inlineStr">
         <is>
@@ -22214,44 +22310,24 @@
         </is>
       </c>
       <c r="K332" t="inlineStr"/>
-      <c r="L332" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="M332" t="n">
-        <v>0</v>
-      </c>
+      <c r="L332" t="inlineStr"/>
+      <c r="M332" t="inlineStr"/>
       <c r="N332" t="n">
-        <v>749177</v>
-      </c>
-      <c r="O332" t="n">
-        <v>1896874</v>
-      </c>
-      <c r="P332" t="n">
-        <v>6.3</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O332" t="inlineStr"/>
+      <c r="P332" t="inlineStr"/>
       <c r="Q332" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="R332" t="n">
-        <v>6.3</v>
-      </c>
+        <v>1849</v>
+      </c>
+      <c r="R332" t="inlineStr"/>
       <c r="S332" t="inlineStr"/>
       <c r="T332" t="inlineStr"/>
-      <c r="U332" t="n">
-        <v>1.708541506212818e-05</v>
-      </c>
-      <c r="V332" t="n">
-        <v>6.747944249328105e-06</v>
-      </c>
-      <c r="W332" t="n">
-        <v>8.409227725891211e-06</v>
-      </c>
-      <c r="X332" t="n">
-        <v>0.3949534866311626</v>
-      </c>
-      <c r="Y332" t="n">
-        <v>0.873015873015873</v>
-      </c>
+      <c r="U332" t="inlineStr"/>
+      <c r="V332" t="inlineStr"/>
+      <c r="W332" t="inlineStr"/>
+      <c r="X332" t="inlineStr"/>
+      <c r="Y332" t="inlineStr"/>
       <c r="Z332" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/sonatel</t>
@@ -22271,34 +22347,48 @@
       <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr">
         <is>
-          <t>missing_report</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>nearest_report_is_different_fiscal_year</t>
+          <t>partial_core_metrics</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>fy=2022 pub=None title=SONATEL SENEGAL : Résultats financiers exercice 2022 [score=60]; fy=2020 pub=None title=SONATEL SENEGAL : Résultats financiers 2020 (Annule et remplace le précédent) [score=60]; fy=2020 pub=None title=SONATEL SENEGAL : Résultats financiers 2020 [score=60]</t>
+          <t>core_metrics_count=2; report=SONATEL SENEGAL : Rapport de gestion exercice 2021</t>
         </is>
       </c>
       <c r="H333" t="n">
-        <v>0</v>
-      </c>
-      <c r="I333" t="inlineStr"/>
-      <c r="J333" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>SONATEL SENEGAL : Rapport de gestion exercice 2021</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/fr/sonatel-senegal-rapport-de-gestion-exercice-2021</t>
+        </is>
+      </c>
       <c r="K333" t="inlineStr"/>
-      <c r="L333" t="inlineStr"/>
-      <c r="M333" t="inlineStr"/>
+      <c r="L333" t="n">
+        <v>25400000000</v>
+      </c>
+      <c r="M333" t="n">
+        <v>862.2</v>
+      </c>
       <c r="N333" t="inlineStr"/>
       <c r="O333" t="inlineStr"/>
       <c r="P333" t="inlineStr"/>
       <c r="Q333" t="inlineStr"/>
       <c r="R333" t="inlineStr"/>
       <c r="S333" t="inlineStr"/>
-      <c r="T333" t="inlineStr"/>
+      <c r="T333" t="n">
+        <v>29459522.1526328</v>
+      </c>
       <c r="U333" t="inlineStr"/>
       <c r="V333" t="inlineStr"/>
       <c r="W333" t="inlineStr"/>
@@ -22343,25 +22433,25 @@
       </c>
       <c r="K334" t="inlineStr"/>
       <c r="L334" t="n">
-        <v>278912</v>
+        <v>278912000000000</v>
       </c>
       <c r="M334" t="n">
         <v>0</v>
       </c>
       <c r="N334" t="n">
-        <v>898523</v>
+        <v>898523000000000</v>
       </c>
       <c r="O334" t="n">
-        <v>2252192</v>
+        <v>2252192000000000</v>
       </c>
       <c r="P334" t="n">
-        <v>294938</v>
+        <v>294938000000000</v>
       </c>
       <c r="Q334" t="n">
-        <v>-66301</v>
+        <v>-66301000000000</v>
       </c>
       <c r="R334" t="n">
-        <v>294938</v>
+        <v>294938000000000</v>
       </c>
       <c r="S334" t="inlineStr"/>
       <c r="T334" t="inlineStr"/>
@@ -22375,10 +22465,10 @@
         <v>0.3282475796390298</v>
       </c>
       <c r="X334" t="n">
-        <v>0.3989548848410793</v>
+        <v>0.3989548848410792</v>
       </c>
       <c r="Y334" t="n">
-        <v>-0.2247963978870136</v>
+        <v>-0.2247963978870135</v>
       </c>
       <c r="Z334" t="inlineStr">
         <is>
@@ -22425,25 +22515,25 @@
       </c>
       <c r="K335" t="inlineStr"/>
       <c r="L335" t="n">
-        <v>331748328</v>
+        <v>3.31748328e+17</v>
       </c>
       <c r="M335" t="n">
         <v>0</v>
       </c>
       <c r="N335" t="n">
-        <v>1065723946</v>
+        <v>1.065723946e+18</v>
       </c>
       <c r="O335" t="n">
-        <v>2573857947</v>
+        <v>2.573857947e+18</v>
       </c>
       <c r="P335" t="n">
-        <v>406102879</v>
+        <v>4.06102879e+17</v>
       </c>
       <c r="Q335" t="n">
-        <v>375015678</v>
+        <v>3.75015678e+17</v>
       </c>
       <c r="R335" t="n">
-        <v>406102879</v>
+        <v>4.06102879e+17</v>
       </c>
       <c r="S335" t="inlineStr"/>
       <c r="T335" t="inlineStr"/>
@@ -22451,7 +22541,7 @@
         <v>0.3112891750674804</v>
       </c>
       <c r="V335" t="n">
-        <v>0.1288914675289965</v>
+        <v>0.1288914675289964</v>
       </c>
       <c r="W335" t="n">
         <v>0.3810582285630654</v>
@@ -22506,34 +22596,34 @@
         </is>
       </c>
       <c r="K336" t="n">
-        <v>619524</v>
+        <v>619524000000000</v>
       </c>
       <c r="L336" t="n">
-        <v>393662</v>
+        <v>393662000000000</v>
       </c>
       <c r="M336" t="n">
-        <v>1776443</v>
+        <v>1776443000000000</v>
       </c>
       <c r="N336" t="n">
-        <v>1274638</v>
+        <v>1274638000000000</v>
       </c>
       <c r="O336" t="n">
-        <v>3105287</v>
+        <v>3105287000000000</v>
       </c>
       <c r="P336" t="n">
-        <v>510764</v>
+        <v>510764000000000</v>
       </c>
       <c r="Q336" t="n">
-        <v>512760</v>
+        <v>512760000000000</v>
       </c>
       <c r="R336" t="n">
-        <v>510764</v>
+        <v>510764000000000</v>
       </c>
       <c r="S336" t="n">
         <v>0.3487440914231416</v>
       </c>
       <c r="T336" t="n">
-        <v>0.2216012559930153</v>
+        <v>0.2216012559930152</v>
       </c>
       <c r="U336" t="n">
         <v>0.3088421967648854</v>
@@ -22593,42 +22683,40 @@
           <t>https://www.brvm.org/sites/default/files/20260216_-_etats_financiers_2025_et_attestation_des_cac_-_sonatel_sn.pdf</t>
         </is>
       </c>
-      <c r="K337" t="inlineStr"/>
+      <c r="K337" t="n">
+        <v>669792000000</v>
+      </c>
       <c r="L337" t="n">
-        <v>413588</v>
-      </c>
-      <c r="M337" t="inlineStr"/>
+        <v>413588000000</v>
+      </c>
+      <c r="M337" t="n">
+        <v>1923122000000</v>
+      </c>
       <c r="N337" t="n">
         <v>1399263</v>
       </c>
-      <c r="O337" t="n">
-        <v>3270175</v>
-      </c>
-      <c r="P337" t="n">
-        <v>643856</v>
-      </c>
+      <c r="O337" t="inlineStr"/>
+      <c r="P337" t="inlineStr"/>
       <c r="Q337" t="n">
-        <v>657038</v>
+        <v>1644154</v>
       </c>
       <c r="R337" t="n">
-        <v>643856</v>
-      </c>
-      <c r="S337" t="inlineStr"/>
-      <c r="T337" t="inlineStr"/>
+        <v>1567737</v>
+      </c>
+      <c r="S337" t="n">
+        <v>0.3482836762306292</v>
+      </c>
+      <c r="T337" t="n">
+        <v>0.2150607189767472</v>
+      </c>
       <c r="U337" t="n">
-        <v>0.2955755994405627</v>
-      </c>
-      <c r="V337" t="n">
-        <v>0.1264727422844343</v>
-      </c>
-      <c r="W337" t="n">
-        <v>0.4601393733701241</v>
-      </c>
-      <c r="X337" t="n">
-        <v>0.4278862751993395</v>
-      </c>
+        <v>295575.5994405627</v>
+      </c>
+      <c r="V337" t="inlineStr"/>
+      <c r="W337" t="inlineStr"/>
+      <c r="X337" t="inlineStr"/>
       <c r="Y337" t="n">
-        <v>1.020473522029771</v>
+        <v>1.048743507361247</v>
       </c>
       <c r="Z337" t="inlineStr">
         <is>
@@ -23061,43 +23149,79 @@
       <c r="B343" t="n">
         <v>2025</v>
       </c>
-      <c r="C343" t="inlineStr"/>
-      <c r="D343" t="inlineStr"/>
+      <c r="C343" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F343" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G343" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=SUCRIVOIRE CÔTE D'IVOIRE : Etats financiers - Normes SYSCOHADA - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr"/>
+      <c r="G343" t="inlineStr"/>
       <c r="H343" t="n">
-        <v>0</v>
-      </c>
-      <c r="I343" t="inlineStr"/>
-      <c r="J343" t="inlineStr"/>
-      <c r="K343" t="inlineStr"/>
-      <c r="L343" t="inlineStr"/>
-      <c r="M343" t="inlineStr"/>
-      <c r="N343" t="inlineStr"/>
-      <c r="O343" t="inlineStr"/>
-      <c r="P343" t="inlineStr"/>
-      <c r="Q343" t="inlineStr"/>
-      <c r="R343" t="inlineStr"/>
-      <c r="S343" t="inlineStr"/>
-      <c r="T343" t="inlineStr"/>
-      <c r="U343" t="inlineStr"/>
-      <c r="V343" t="inlineStr"/>
-      <c r="W343" t="inlineStr"/>
-      <c r="X343" t="inlineStr"/>
-      <c r="Y343" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>SUCRIVOIRE CI : Etats financiers SYSCOHADA - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260430_-_etats_financiers_syscohada_-_exercice_2025_-_sucrivoire_ci.pdf</t>
+        </is>
+      </c>
+      <c r="K343" t="n">
+        <v>1828947146</v>
+      </c>
+      <c r="L343" t="n">
+        <v>6131800226</v>
+      </c>
+      <c r="M343" t="n">
+        <v>8</v>
+      </c>
+      <c r="N343" t="n">
+        <v>13822035189</v>
+      </c>
+      <c r="O343" t="n">
+        <v>83125331794</v>
+      </c>
+      <c r="P343" t="n">
+        <v>69303296605</v>
+      </c>
+      <c r="Q343" t="n">
+        <v>59213082787</v>
+      </c>
+      <c r="R343" t="n">
+        <v>52902913471</v>
+      </c>
+      <c r="S343" t="n">
+        <v>228618393.25</v>
+      </c>
+      <c r="T343" t="n">
+        <v>766475028.25</v>
+      </c>
+      <c r="U343" t="n">
+        <v>0.4436249902532353</v>
+      </c>
+      <c r="V343" t="n">
+        <v>0.07376572332000718</v>
+      </c>
+      <c r="W343" t="n">
+        <v>5.013971940988379</v>
+      </c>
+      <c r="X343" t="n">
+        <v>0.1662794588688508</v>
+      </c>
+      <c r="Y343" t="n">
+        <v>1.119278294936612</v>
+      </c>
       <c r="Z343" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/sucrivoire</t>
@@ -25297,7 +25421,7 @@
       <c r="F385" t="inlineStr"/>
       <c r="G385" t="inlineStr"/>
       <c r="H385" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I385" t="inlineStr">
         <is>
@@ -25318,42 +25442,28 @@
       <c r="M385" t="n">
         <v>588709</v>
       </c>
-      <c r="N385" t="n">
-        <v>36202</v>
-      </c>
+      <c r="N385" t="inlineStr"/>
       <c r="O385" t="n">
-        <v>342925</v>
-      </c>
-      <c r="P385" t="n">
-        <v>306723</v>
-      </c>
+        <v>188472191526</v>
+      </c>
+      <c r="P385" t="inlineStr"/>
       <c r="Q385" t="n">
-        <v>108382</v>
-      </c>
-      <c r="R385" t="n">
-        <v>118044</v>
-      </c>
+        <v>108382106956</v>
+      </c>
+      <c r="R385" t="inlineStr"/>
       <c r="S385" t="n">
-        <v>0.0209424350570485</v>
+        <v>0.02094243505704856</v>
       </c>
       <c r="T385" t="n">
-        <v>0.015435469816157</v>
-      </c>
-      <c r="U385" t="n">
-        <v>0.2510082315894149</v>
-      </c>
+        <v>0.01543546981615705</v>
+      </c>
+      <c r="U385" t="inlineStr"/>
       <c r="V385" t="n">
-        <v>0.0264985055041189</v>
-      </c>
-      <c r="W385" t="n">
-        <v>8.472542953427988</v>
-      </c>
-      <c r="X385" t="n">
-        <v>0.1055682729459794</v>
-      </c>
-      <c r="Y385" t="n">
-        <v>0.9181491647182408</v>
-      </c>
+        <v>4.821400932639145e-08</v>
+      </c>
+      <c r="W385" t="inlineStr"/>
+      <c r="X385" t="inlineStr"/>
+      <c r="Y385" t="inlineStr"/>
       <c r="Z385" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/total</t>
@@ -25378,10 +25488,14 @@
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>no_reports_found_on_company_page</t>
-        </is>
-      </c>
-      <c r="G386" t="inlineStr"/>
+          <t>no_candidate_for_fiscal_year</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>fy=2024 pub=2025 title=TOTALENERGIES MARKETING SN : Etats financiers IFRS - Exercice 2024 [score=260]; fy=2025 pub=2026 title=TOTALENERGIES MARKETING SN : Etats financiers SYSCOHADA - Exercice 2025 [score=260]</t>
+        </is>
+      </c>
       <c r="H386" t="n">
         <v>0</v>
       </c>
@@ -25426,10 +25540,14 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>no_reports_found_on_company_page</t>
-        </is>
-      </c>
-      <c r="G387" t="inlineStr"/>
+          <t>no_candidate_for_fiscal_year</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>fy=2024 pub=2025 title=TOTALENERGIES MARKETING SN : Etats financiers IFRS - Exercice 2024 [score=260]; fy=2025 pub=2026 title=TOTALENERGIES MARKETING SN : Etats financiers SYSCOHADA - Exercice 2025 [score=260]</t>
+        </is>
+      </c>
       <c r="H387" t="n">
         <v>0</v>
       </c>
@@ -25474,10 +25592,14 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>no_reports_found_on_company_page</t>
-        </is>
-      </c>
-      <c r="G388" t="inlineStr"/>
+          <t>no_candidate_for_fiscal_year</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>fy=2024 pub=2025 title=TOTALENERGIES MARKETING SN : Etats financiers IFRS - Exercice 2024 [score=260]; fy=2025 pub=2026 title=TOTALENERGIES MARKETING SN : Etats financiers SYSCOHADA - Exercice 2025 [score=260]</t>
+        </is>
+      </c>
       <c r="H388" t="n">
         <v>0</v>
       </c>
@@ -25522,10 +25644,14 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>no_reports_found_on_company_page</t>
-        </is>
-      </c>
-      <c r="G389" t="inlineStr"/>
+          <t>nearest_report_is_different_fiscal_year</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>fy=2024 pub=2025 title=TOTALENERGIES MARKETING SN : Etats financiers IFRS - Exercice 2024 [score=260]</t>
+        </is>
+      </c>
       <c r="H389" t="n">
         <v>0</v>
       </c>
@@ -25561,39 +25687,79 @@
       <c r="B390" t="n">
         <v>2024</v>
       </c>
-      <c r="C390" t="inlineStr"/>
-      <c r="D390" t="inlineStr"/>
+      <c r="C390" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>2025-05-02</t>
+        </is>
+      </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F390" t="inlineStr">
-        <is>
-          <t>no_reports_found_on_company_page</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr"/>
       <c r="G390" t="inlineStr"/>
       <c r="H390" t="n">
-        <v>0</v>
-      </c>
-      <c r="I390" t="inlineStr"/>
-      <c r="J390" t="inlineStr"/>
-      <c r="K390" t="inlineStr"/>
-      <c r="L390" t="inlineStr"/>
-      <c r="M390" t="inlineStr"/>
-      <c r="N390" t="inlineStr"/>
-      <c r="O390" t="inlineStr"/>
-      <c r="P390" t="inlineStr"/>
-      <c r="Q390" t="inlineStr"/>
-      <c r="R390" t="inlineStr"/>
-      <c r="S390" t="inlineStr"/>
-      <c r="T390" t="inlineStr"/>
-      <c r="U390" t="inlineStr"/>
-      <c r="V390" t="inlineStr"/>
-      <c r="W390" t="inlineStr"/>
-      <c r="X390" t="inlineStr"/>
-      <c r="Y390" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>TOTALENERGIES MARKETING SN : Etats financiers IFRS - Exercice 2024</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20250502_-_etats_financiers_-_norme_ifrs_-_exercice_2024_-_totalenergies_marketing_sn.pdf</t>
+        </is>
+      </c>
+      <c r="K390" t="n">
+        <v>7208</v>
+      </c>
+      <c r="L390" t="n">
+        <v>7140</v>
+      </c>
+      <c r="M390" t="n">
+        <v>484945</v>
+      </c>
+      <c r="N390" t="n">
+        <v>26911</v>
+      </c>
+      <c r="O390" t="n">
+        <v>210418</v>
+      </c>
+      <c r="P390" t="n">
+        <v>183507</v>
+      </c>
+      <c r="Q390" t="n">
+        <v>150004</v>
+      </c>
+      <c r="R390" t="n">
+        <v>178126</v>
+      </c>
+      <c r="S390" t="n">
+        <v>0.0148635412263246</v>
+      </c>
+      <c r="T390" t="n">
+        <v>0.0147233191392838</v>
+      </c>
+      <c r="U390" t="n">
+        <v>0.2653190145293746</v>
+      </c>
+      <c r="V390" t="n">
+        <v>0.0339324582497695</v>
+      </c>
+      <c r="W390" t="n">
+        <v>6.819033109137528</v>
+      </c>
+      <c r="X390" t="n">
+        <v>0.1278930509747265</v>
+      </c>
+      <c r="Y390" t="n">
+        <v>0.8421229915902226</v>
+      </c>
       <c r="Z390" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/total-senegal-sa</t>
@@ -25609,39 +25775,79 @@
       <c r="B391" t="n">
         <v>2025</v>
       </c>
-      <c r="C391" t="inlineStr"/>
-      <c r="D391" t="inlineStr"/>
+      <c r="C391" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F391" t="inlineStr">
-        <is>
-          <t>no_reports_found_on_company_page</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr"/>
       <c r="H391" t="n">
-        <v>0</v>
-      </c>
-      <c r="I391" t="inlineStr"/>
-      <c r="J391" t="inlineStr"/>
-      <c r="K391" t="inlineStr"/>
-      <c r="L391" t="inlineStr"/>
-      <c r="M391" t="inlineStr"/>
-      <c r="N391" t="inlineStr"/>
-      <c r="O391" t="inlineStr"/>
-      <c r="P391" t="inlineStr"/>
-      <c r="Q391" t="inlineStr"/>
-      <c r="R391" t="inlineStr"/>
-      <c r="S391" t="inlineStr"/>
-      <c r="T391" t="inlineStr"/>
-      <c r="U391" t="inlineStr"/>
-      <c r="V391" t="inlineStr"/>
-      <c r="W391" t="inlineStr"/>
-      <c r="X391" t="inlineStr"/>
-      <c r="Y391" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>TOTALENERGIES MARKETING SN : Etats financiers SYSCOHADA - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260430_-_etats_financiers_syscohada_-_exercice_2025_-_totalenergies_marketing_sn.pdf</t>
+        </is>
+      </c>
+      <c r="K391" t="n">
+        <v>7880032</v>
+      </c>
+      <c r="L391" t="n">
+        <v>6146527</v>
+      </c>
+      <c r="M391" t="n">
+        <v>455208888</v>
+      </c>
+      <c r="N391" t="n">
+        <v>41679</v>
+      </c>
+      <c r="O391" t="n">
+        <v>158397943</v>
+      </c>
+      <c r="P391" t="n">
+        <v>133684057</v>
+      </c>
+      <c r="Q391" t="n">
+        <v>114800736</v>
+      </c>
+      <c r="R391" t="n">
+        <v>124515903</v>
+      </c>
+      <c r="S391" t="n">
+        <v>0.01731080435318741</v>
+      </c>
+      <c r="T391" t="n">
+        <v>0.01350265155631144</v>
+      </c>
+      <c r="U391" t="n">
+        <v>147.472995993186</v>
+      </c>
+      <c r="V391" t="n">
+        <v>0.03880433598812581</v>
+      </c>
+      <c r="W391" t="n">
+        <v>3207.467957484585</v>
+      </c>
+      <c r="X391" t="n">
+        <v>0.0002631284170148598</v>
+      </c>
+      <c r="Y391" t="n">
+        <v>0.9219764964480079</v>
+      </c>
       <c r="Z391" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/total-senegal-sa</t>
@@ -26913,38 +27119,62 @@
       <c r="B415" t="n">
         <v>2025</v>
       </c>
-      <c r="C415" t="inlineStr"/>
-      <c r="D415" t="inlineStr"/>
+      <c r="C415" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>missing_report</t>
-        </is>
-      </c>
-      <c r="F415" t="inlineStr">
-        <is>
-          <t>nearest_report_is_different_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G415" t="inlineStr">
-        <is>
-          <t>fy=2024 pub=2025 title=TRACTAFRIC MOTORS CÔTE D'IVOIRE : Etats financiers - Normes IFRS - Exercice 2024 [score=60]</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr"/>
+      <c r="G415" t="inlineStr"/>
       <c r="H415" t="n">
-        <v>0</v>
-      </c>
-      <c r="I415" t="inlineStr"/>
-      <c r="J415" t="inlineStr"/>
-      <c r="K415" t="inlineStr"/>
-      <c r="L415" t="inlineStr"/>
-      <c r="M415" t="inlineStr"/>
-      <c r="N415" t="inlineStr"/>
-      <c r="O415" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>TRACTAFRIC MOTORS CI : Etats financiers - Exercice 2025</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>https://www.brvm.org/sites/default/files/20260430_-_etats_financiers_-_exercice_2025_-_tractafric_motors_ci.pdf</t>
+        </is>
+      </c>
+      <c r="K415" t="n">
+        <v>4240878619</v>
+      </c>
+      <c r="L415" t="n">
+        <v>0</v>
+      </c>
+      <c r="M415" t="n">
+        <v>81126957415</v>
+      </c>
+      <c r="N415" t="n">
+        <v>0</v>
+      </c>
+      <c r="O415" t="n">
+        <v>0</v>
+      </c>
       <c r="P415" t="inlineStr"/>
-      <c r="Q415" t="inlineStr"/>
-      <c r="R415" t="inlineStr"/>
-      <c r="S415" t="inlineStr"/>
-      <c r="T415" t="inlineStr"/>
+      <c r="Q415" t="n">
+        <v>0</v>
+      </c>
+      <c r="R415" t="n">
+        <v>0</v>
+      </c>
+      <c r="S415" t="n">
+        <v>0.05227459224565818</v>
+      </c>
+      <c r="T415" t="n">
+        <v>0</v>
+      </c>
       <c r="U415" t="inlineStr"/>
       <c r="V415" t="inlineStr"/>
       <c r="W415" t="inlineStr"/>
@@ -27662,14 +27892,10 @@
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G427" t="inlineStr">
-        <is>
-          <t>fy=2021 pub=2022 title=UNILEVER CI : Etats financiers Exercice 2021 [score=60]; fy=2020 pub=2021 title=UNILEVER CÔTE D'IVOIRE : Etats Financiers - Exercice 2020 [score=60]; fy=2023 pub=2024 title=UNILEVER CÔTE D'IVOIRE : Etats Financiers - Exercice 2023 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr"/>
       <c r="H427" t="n">
         <v>0</v>
       </c>
@@ -28301,11 +28527,11 @@
       <c r="F435" t="inlineStr"/>
       <c r="G435" t="inlineStr"/>
       <c r="H435" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t>VIVO ENERGY CI : Etats Financiers exercice 2021</t>
+          <t>VIVO ENERGY CI : Etats financiers exercice 2021</t>
         </is>
       </c>
       <c r="J435" t="inlineStr">
@@ -28320,44 +28546,28 @@
         <v>2359622661</v>
       </c>
       <c r="M435" t="n">
-        <v>366643579663</v>
-      </c>
-      <c r="N435" t="n">
-        <v>500376822</v>
-      </c>
+        <v>3.666435796633136e+23</v>
+      </c>
+      <c r="N435" t="inlineStr"/>
       <c r="O435" t="n">
         <v>101262735128</v>
       </c>
-      <c r="P435" t="n">
-        <v>67133730036</v>
-      </c>
-      <c r="Q435" t="n">
-        <v>43810997944</v>
-      </c>
-      <c r="R435" t="n">
-        <v>48939413906</v>
-      </c>
+      <c r="P435" t="inlineStr"/>
+      <c r="Q435" t="inlineStr"/>
+      <c r="R435" t="inlineStr"/>
       <c r="S435" t="n">
-        <v>0.011643192868463</v>
+        <v>1.164319286845308e-14</v>
       </c>
       <c r="T435" t="n">
-        <v>0.0064357397534926</v>
-      </c>
-      <c r="U435" t="n">
-        <v>4.71569136949353</v>
-      </c>
+        <v>6.435739753487096e-15</v>
+      </c>
+      <c r="U435" t="inlineStr"/>
       <c r="V435" t="n">
         <v>0.0233019842691128</v>
       </c>
-      <c r="W435" t="n">
-        <v>134.1663464100262</v>
-      </c>
-      <c r="X435" t="n">
-        <v>0.0049413717826948</v>
-      </c>
-      <c r="Y435" t="n">
-        <v>0.8952088806815226</v>
-      </c>
+      <c r="W435" t="inlineStr"/>
+      <c r="X435" t="inlineStr"/>
+      <c r="Y435" t="inlineStr"/>
       <c r="Z435" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/vivo-energy-ci</t>
@@ -28389,7 +28599,7 @@
       <c r="F436" t="inlineStr"/>
       <c r="G436" t="inlineStr"/>
       <c r="H436" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I436" t="inlineStr">
         <is>
@@ -28402,50 +28612,34 @@
         </is>
       </c>
       <c r="K436" t="n">
-        <v>4363474241</v>
+        <v>6027152226</v>
       </c>
       <c r="L436" t="n">
         <v>3548638458</v>
       </c>
       <c r="M436" t="n">
-        <v>488901792280</v>
-      </c>
-      <c r="N436" t="n">
-        <v>3548638458</v>
-      </c>
+        <v>4.889017922803666e+35</v>
+      </c>
+      <c r="N436" t="inlineStr"/>
       <c r="O436" t="n">
-        <v>119461700193</v>
-      </c>
-      <c r="P436" t="n">
-        <v>96547661925</v>
-      </c>
-      <c r="Q436" t="n">
-        <v>59723429880</v>
-      </c>
-      <c r="R436" t="n">
-        <v>79528604069</v>
-      </c>
+        <v>1.194617001931013e+23</v>
+      </c>
+      <c r="P436" t="inlineStr"/>
+      <c r="Q436" t="inlineStr"/>
+      <c r="R436" t="inlineStr"/>
       <c r="S436" t="n">
-        <v>0.008925052658634899</v>
+        <v>1.232794054177584e-26</v>
       </c>
       <c r="T436" t="n">
-        <v>0.0072583870913028</v>
-      </c>
-      <c r="U436" t="n">
-        <v>1</v>
-      </c>
+        <v>7.25838709129745e-27</v>
+      </c>
+      <c r="U436" t="inlineStr"/>
       <c r="V436" t="n">
-        <v>0.0297052398573508</v>
-      </c>
-      <c r="W436" t="n">
-        <v>27.2069592514685</v>
-      </c>
-      <c r="X436" t="n">
-        <v>0.0297052398573508</v>
-      </c>
-      <c r="Y436" t="n">
-        <v>0.7509679137355814</v>
-      </c>
+        <v>2.970523985732566e-14</v>
+      </c>
+      <c r="W436" t="inlineStr"/>
+      <c r="X436" t="inlineStr"/>
+      <c r="Y436" t="inlineStr"/>
       <c r="Z436" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/vivo-energy-ci</t>
@@ -28477,7 +28671,7 @@
       <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr"/>
       <c r="H437" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I437" t="inlineStr">
         <is>
@@ -28490,50 +28684,34 @@
         </is>
       </c>
       <c r="K437" t="n">
-        <v>8485512286</v>
+        <v>41</v>
       </c>
       <c r="L437" t="n">
         <v>4011602748</v>
       </c>
       <c r="M437" t="n">
-        <v>550696</v>
-      </c>
-      <c r="N437" t="n">
-        <v>7161602748</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="N437" t="inlineStr"/>
       <c r="O437" t="n">
-        <v>168468608785</v>
-      </c>
-      <c r="P437" t="n">
-        <v>51213273269</v>
-      </c>
-      <c r="Q437" t="n">
-        <v>49890581130</v>
-      </c>
-      <c r="R437" t="n">
-        <v>36104035916</v>
-      </c>
+        <v>1.684686087851195e+23</v>
+      </c>
+      <c r="P437" t="inlineStr"/>
+      <c r="Q437" t="inlineStr"/>
+      <c r="R437" t="inlineStr"/>
       <c r="S437" t="n">
-        <v>15408.70514040414</v>
+        <v>3.153846153846154</v>
       </c>
       <c r="T437" t="n">
-        <v>7284.60484187283</v>
-      </c>
-      <c r="U437" t="n">
-        <v>0.5601543242705425</v>
-      </c>
+        <v>308584826.7692308</v>
+      </c>
+      <c r="U437" t="inlineStr"/>
       <c r="V437" t="n">
-        <v>0.0238121676016189</v>
-      </c>
-      <c r="W437" t="n">
-        <v>7.151091043593864</v>
-      </c>
-      <c r="X437" t="n">
-        <v>0.0425100129908453</v>
-      </c>
-      <c r="Y437" t="n">
-        <v>1.381856068559092</v>
-      </c>
+        <v>2.38121676016021e-14</v>
+      </c>
+      <c r="W437" t="inlineStr"/>
+      <c r="X437" t="inlineStr"/>
+      <c r="Y437" t="inlineStr"/>
       <c r="Z437" t="inlineStr">
         <is>
           <t>https://www.brvm.org/fr/rapports-societe-cotes/vivo-energy-ci</t>
@@ -28610,14 +28788,10 @@
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>no_candidate_for_fiscal_year</t>
-        </is>
-      </c>
-      <c r="G439" t="inlineStr">
-        <is>
-          <t>fy=2023 pub=2024 title=VIVO ENERGY CI : Etats Financiers provisoire - Exercice 2023 [score=70]; fy=2023 pub=2024 title=VIVO ENERGY CI : Etats Financiers provisoire 2023 [score=70]; fy=2022 pub=2023 title=VIVO ENERGY : Etats financiers - Exercice 2022 [score=60]</t>
-        </is>
-      </c>
+          <t>no_reports_found_on_company_page</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr"/>
       <c r="H439" t="n">
         <v>0</v>
       </c>

</xml_diff>